<commit_message>
testing worfklow for get weather
</commit_message>
<xml_diff>
--- a/BOOKING_RESULT_Brasov_15_May_2026_20_July_2026_3_guests.xlsx
+++ b/BOOKING_RESULT_Brasov_15_May_2026_20_July_2026_3_guests.xlsx
@@ -37,6 +37,78 @@
     <x:t>1</x:t>
   </x:si>
   <x:si>
+    <x:t>Standard Suite</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ONE66 - Luxury Aparthotel</x:t>
+  </x:si>
+  <x:si>
+    <x:t>182.76</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9.3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/one66.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=1&amp;hapos=1&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=1391861902_411156230_3_0_0_1199065&amp;highlighted_blocks=1391861902_411156230_3_0_0_1199065&amp;matching_block_id=1391861902_411156230_3_0_0_1199065&amp;sr_pri_blocks=1391861902_411156230_3_0_0_1199065_6138634&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t/>
+  </x:si>
+  <x:si>
+    <x:t>Hotel Rainer</x:t>
+  </x:si>
+  <x:si>
+    <x:t>145.67</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8.6</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/rainer.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=2&amp;hapos=2&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=17959202_424251257_2_1_0%2C17959202_424251257_2_1_0&amp;highlighted_blocks=17959202_424251257_2_1_0%2C17959202_424251257_2_1_0&amp;matching_block_id=17959202_424251257_2_1_0&amp;sr_pri_blocks=17959202_424251257_2_1_0__2446290%2C17959202_424251257_2_1_0__2446290&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Deluxe Suite</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Muresenilor 9 Boutique - Old Town</x:t>
+  </x:si>
+  <x:si>
+    <x:t>137.08</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9.4</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/muresenilor-9.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=3&amp;hapos=3&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=1324526603_405092771_3_0_0&amp;highlighted_blocks=1324526603_405092771_3_0_0&amp;matching_block_id=1324526603_405092771_3_0_0&amp;sr_pri_blocks=1324526603_405092771_3_0_0__4604300&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Deluxe Suite upper floors no elevator</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Casa Cranta</x:t>
+  </x:si>
+  <x:si>
+    <x:t>141.79</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9.2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/casa-cranta.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=4&amp;hapos=4&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=4607605_178126435_3_2_0&amp;highlighted_blocks=4607605_178126435_3_2_0&amp;matching_block_id=4607605_178126435_3_2_0&amp;sr_pri_blocks=4607605_178126435_3_2_0__4762300&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Family Suite</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Belfort Hotel</x:t>
+  </x:si>
+  <x:si>
+    <x:t>197.86</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/belfort-hotel.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=5&amp;hapos=5&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=4740913_129959805_3_1_0_495792&amp;highlighted_blocks=4740913_129959805_3_1_0_495792&amp;matching_block_id=4740913_129959805_3_1_0_495792&amp;sr_pri_blocks=4740913_129959805_3_1_0_495792_6646200&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
     <x:t>Triple Room</x:t>
   </x:si>
   <x:si>
@@ -46,10 +118,67 @@
     <x:t>90.5</x:t>
   </x:si>
   <x:si>
-    <x:t>9.2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/bark-inn-bed-and-breakfast.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=1&amp;hapos=1&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=1320902003_404782112_0_1_0&amp;highlighted_blocks=1320902003_404782112_0_1_0&amp;matching_block_id=1320902003_404782112_0_1_0&amp;sr_pri_blocks=1320902003_404782112_0_1_0__3039966&amp;from=searchresults</x:t>
+    <x:t>https://www.booking.com/hotel/ro/bark-inn-bed-and-breakfast.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=6&amp;hapos=6&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=1320902003_404782112_0_1_0&amp;highlighted_blocks=1320902003_404782112_0_1_0&amp;matching_block_id=1320902003_404782112_0_1_0&amp;sr_pri_blocks=1320902003_404782112_0_1_0__3039966&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Deluxe Family Suite</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Vila William’s</x:t>
+  </x:si>
+  <x:si>
+    <x:t>86.77</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/vila-williams.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=7&amp;hapos=7&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=435337304_147308954_0_0_0_874904&amp;highlighted_blocks=435337304_147308954_0_0_0_874904&amp;matching_block_id=435337304_147308954_0_0_0_874904&amp;sr_pri_blocks=435337304_147308954_0_0_0_874904_2914560&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Two-Bedroom Apartment with Terrace</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Relax in Style Boutique Hotel</x:t>
+  </x:si>
+  <x:si>
+    <x:t>168.29</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8.1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/villa-in-style.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=8&amp;hapos=8&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=791352814_417023336_3_0_0_869436&amp;highlighted_blocks=791352814_417023336_3_0_0_869436&amp;matching_block_id=791352814_417023336_3_0_0_869436&amp;sr_pri_blocks=791352814_417023336_3_0_0_869436_5652600&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ALBERT RESIDENCE Brasov with complimentary parking off site</x:t>
+  </x:si>
+  <x:si>
+    <x:t>370.58</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/albert-residence.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=9&amp;hapos=9&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=722324407_309584935_2_1_0%2C722324408_309584935_1_1_0&amp;highlighted_blocks=722324407_309584935_2_1_0%2C722324408_309584935_1_1_0&amp;matching_block_id=722324407_309584935_2_1_0&amp;sr_pri_blocks=722324407_309584935_2_1_0__6584610%2C722324408_309584935_1_1_0__5862789&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Deluxe Apartment</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HOTEL BOUTIQUE CASA CHITIC -HOTEL AND RESTAURANT Str Johann Gott nr7</x:t>
+  </x:si>
+  <x:si>
+    <x:t>208.68</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/casa-chitic.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=10&amp;hapos=10&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=356850201_131980679_0_1_0&amp;highlighted_blocks=356850201_131980679_0_1_0&amp;matching_block_id=356850201_131980679_0_1_0&amp;sr_pri_blocks=356850201_131980679_0_1_0__7009200&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Hotel Brasov</x:t>
+  </x:si>
+  <x:si>
+    <x:t>160.21</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9.0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/brasov.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=11&amp;hapos=11&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=28530702_362275009_0_1_0%2C28530703_362275009_1_1_0&amp;highlighted_blocks=28530702_362275009_0_1_0%2C28530703_362275009_1_1_0&amp;matching_block_id=28530702_362275009_0_1_0&amp;sr_pri_blocks=28530702_362275009_0_1_0__2866816%2C28530703_362275009_1_1_0__2514514&amp;from=searchresults</x:t>
   </x:si>
   <x:si>
     <x:t>One-Bedroom Apartment</x:t>
@@ -61,67 +190,46 @@
     <x:t>91.26</x:t>
   </x:si>
   <x:si>
-    <x:t>9.0</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/peak-aparthotel-by-cityhost.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=2&amp;hapos=2&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=1166912003_389307937_3_0_0&amp;highlighted_blocks=1166912003_389307937_3_0_0&amp;matching_block_id=1166912003_389307937_3_0_0&amp;sr_pri_blocks=1166912003_389307937_3_0_0__3064993&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Standard Suite</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ONE66 - Luxury Aparthotel</x:t>
-  </x:si>
-  <x:si>
-    <x:t>182.76</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9.3</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/one66.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=3&amp;hapos=3&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=1391861902_411156230_3_0_0_1199065&amp;highlighted_blocks=1391861902_411156230_3_0_0_1199065&amp;matching_block_id=1391861902_411156230_3_0_0_1199065&amp;sr_pri_blocks=1391861902_411156230_3_0_0_1199065_6138634&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t/>
-  </x:si>
-  <x:si>
-    <x:t>Hotel Rainer</x:t>
-  </x:si>
-  <x:si>
-    <x:t>145.67</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8.6</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/rainer.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=4&amp;hapos=4&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=17959202_424251257_2_1_0%2C17959202_424251257_2_1_0&amp;highlighted_blocks=17959202_424251257_2_1_0%2C17959202_424251257_2_1_0&amp;matching_block_id=17959202_424251257_2_1_0&amp;sr_pri_blocks=17959202_424251257_2_1_0__2446290%2C17959202_424251257_2_1_0__2446290&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Deluxe Suite</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Muresenilor 9 Boutique - Old Town</x:t>
-  </x:si>
-  <x:si>
-    <x:t>137.08</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9.4</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/muresenilor-9.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=5&amp;hapos=5&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=1324526603_405092771_3_0_0&amp;highlighted_blocks=1324526603_405092771_3_0_0&amp;matching_block_id=1324526603_405092771_3_0_0&amp;sr_pri_blocks=1324526603_405092771_3_0_0__4604300&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Deluxe Suite upper floors no elevator</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Casa Cranta</x:t>
-  </x:si>
-  <x:si>
-    <x:t>141.79</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/casa-cranta.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=6&amp;hapos=6&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=4607605_178126435_3_2_0&amp;highlighted_blocks=4607605_178126435_3_2_0&amp;matching_block_id=4607605_178126435_3_2_0&amp;sr_pri_blocks=4607605_178126435_3_2_0__4762300&amp;from=searchresults</x:t>
+    <x:t>https://www.booking.com/hotel/ro/peak-aparthotel-by-cityhost.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=12&amp;hapos=12&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=1166912003_389307937_3_0_0&amp;highlighted_blocks=1166912003_389307937_3_0_0&amp;matching_block_id=1166912003_389307937_3_0_0&amp;sr_pri_blocks=1166912003_389307937_3_0_0__3064993&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Deluxe Triple Room with Balcony</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Grand Hotel</x:t>
+  </x:si>
+  <x:si>
+    <x:t>135.5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8.2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/grand.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=13&amp;hapos=13&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=4127217_144025049_3_1_0&amp;highlighted_blocks=4127217_144025049_3_1_0&amp;matching_block_id=4127217_144025049_3_1_0&amp;sr_pri_blocks=4127217_144025049_3_1_0__4551520&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Apart Hotel Vlad Tepes</x:t>
+  </x:si>
+  <x:si>
+    <x:t>197.47</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9.1</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/apart-vlad-tepes.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=14&amp;hapos=14&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=35764301_278507467_2_0_0%2C35764301_278507467_2_0_0&amp;highlighted_blocks=35764301_278507467_2_0_0%2C35764301_278507467_2_0_0&amp;matching_block_id=35764301_278507467_2_0_0&amp;sr_pri_blocks=35764301_278507467_2_0_0__3356100%2C35764301_278507467_2_0_0__3276900&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Family Room</x:t>
+  </x:si>
+  <x:si>
+    <x:t>La Dolce Vita Central</x:t>
+  </x:si>
+  <x:si>
+    <x:t>66.2</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/la-dolce-vita-central.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=15&amp;hapos=15&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=1415864003_413286899_3_2_0&amp;highlighted_blocks=1415864003_413286899_3_2_0&amp;matching_block_id=1415864003_413286899_3_2_0&amp;sr_pri_blocks=1415864003_413286899_3_2_0__2223524&amp;from=searchresults</x:t>
   </x:si>
   <x:si>
     <x:t>Basic Triple Room</x:t>
@@ -136,115 +244,7 @@
     <x:t>8.3</x:t>
   </x:si>
   <x:si>
-    <x:t>https://www.booking.com/hotel/ro/casa-muresan.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=7&amp;hapos=7&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=4137714_128926762_0_2_0&amp;highlighted_blocks=4137714_128926762_0_2_0&amp;matching_block_id=4137714_128926762_0_2_0&amp;sr_pri_blocks=4137714_128926762_0_2_0__2806056&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Deluxe Family Suite</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Vila William’s</x:t>
-  </x:si>
-  <x:si>
-    <x:t>86.77</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/vila-williams.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=8&amp;hapos=8&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=435337304_147308954_0_0_0_874904&amp;highlighted_blocks=435337304_147308954_0_0_0_874904&amp;matching_block_id=435337304_147308954_0_0_0_874904&amp;sr_pri_blocks=435337304_147308954_0_0_0_874904_2914560&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Two-Bedroom Apartment with Terrace</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Relax in Style Boutique Hotel</x:t>
-  </x:si>
-  <x:si>
-    <x:t>168.29</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8.1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/villa-in-style.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=9&amp;hapos=9&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=791352814_417023336_3_0_0_869436&amp;highlighted_blocks=791352814_417023336_3_0_0_869436&amp;matching_block_id=791352814_417023336_3_0_0_869436&amp;sr_pri_blocks=791352814_417023336_3_0_0_869436_5652600&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>ALBERT RESIDENCE Brasov with complimentary parking off site</x:t>
-  </x:si>
-  <x:si>
-    <x:t>334.23</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/albert-residence.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=10&amp;hapos=10&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=722324407_309584935_2_1_0%2C722324408_309584935_1_1_0&amp;highlighted_blocks=722324407_309584935_2_1_0%2C722324408_309584935_1_1_0&amp;matching_block_id=722324407_309584935_2_1_0&amp;sr_pri_blocks=722324407_309584935_2_1_0__5941989%2C722324408_309584935_1_1_0__5284430&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Deluxe Apartment</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HOTEL BOUTIQUE CASA CHITIC -HOTEL AND RESTAURANT Str Johann Gott nr7</x:t>
-  </x:si>
-  <x:si>
-    <x:t>208.68</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/casa-chitic.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=11&amp;hapos=11&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=356850201_131980679_0_1_0&amp;highlighted_blocks=356850201_131980679_0_1_0&amp;matching_block_id=356850201_131980679_0_1_0&amp;sr_pri_blocks=356850201_131980679_0_1_0__7009200&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Hotel Brasov</x:t>
-  </x:si>
-  <x:si>
-    <x:t>160.21</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/brasov.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=12&amp;hapos=12&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=28530702_362275009_0_1_0%2C28530703_362275009_1_1_0&amp;highlighted_blocks=28530702_362275009_0_1_0%2C28530703_362275009_1_1_0&amp;matching_block_id=28530702_362275009_0_1_0&amp;sr_pri_blocks=28530702_362275009_0_1_0__2866816%2C28530703_362275009_1_1_0__2514514&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Deluxe Triple Room with Balcony</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Grand Hotel</x:t>
-  </x:si>
-  <x:si>
-    <x:t>135.5</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8.2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/grand.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=13&amp;hapos=13&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=4127217_144025049_3_1_0&amp;highlighted_blocks=4127217_144025049_3_1_0&amp;matching_block_id=4127217_144025049_3_1_0&amp;sr_pri_blocks=4127217_144025049_3_1_0__4551520&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Apart Hotel Vlad Tepes</x:t>
-  </x:si>
-  <x:si>
-    <x:t>197.47</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9.1</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/apart-vlad-tepes.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=14&amp;hapos=14&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=35764301_278507467_2_0_0%2C35764301_278507467_2_0_0&amp;highlighted_blocks=35764301_278507467_2_0_0%2C35764301_278507467_2_0_0&amp;matching_block_id=35764301_278507467_2_0_0&amp;sr_pri_blocks=35764301_278507467_2_0_0__3356100%2C35764301_278507467_2_0_0__3276900&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Family Room</x:t>
-  </x:si>
-  <x:si>
-    <x:t>La Dolce Vita Central</x:t>
-  </x:si>
-  <x:si>
-    <x:t>66.2</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/la-dolce-vita-central.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=15&amp;hapos=15&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=1415864003_413286899_3_2_0&amp;highlighted_blocks=1415864003_413286899_3_2_0&amp;matching_block_id=1415864003_413286899_3_2_0&amp;sr_pri_blocks=1415864003_413286899_3_2_0__2223524&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Family Suite</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Belfort Hotel</x:t>
-  </x:si>
-  <x:si>
-    <x:t>197.86</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/belfort-hotel.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=16&amp;hapos=16&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=4740913_129959805_3_1_0_495792&amp;highlighted_blocks=4740913_129959805_3_1_0_495792&amp;matching_block_id=4740913_129959805_3_1_0_495792&amp;sr_pri_blocks=4740913_129959805_3_1_0_495792_6646200&amp;from=searchresults</x:t>
+    <x:t>https://www.booking.com/hotel/ro/casa-muresan.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=16&amp;hapos=16&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=4137714_128926762_0_2_0&amp;highlighted_blocks=4137714_128926762_0_2_0&amp;matching_block_id=4137714_128926762_0_2_0&amp;sr_pri_blocks=4137714_128926762_0_2_0__2806056&amp;from=searchresults</x:t>
   </x:si>
   <x:si>
     <x:t>Hotel Jasmine</x:t>
@@ -256,7 +256,7 @@
     <x:t>9.6</x:t>
   </x:si>
   <x:si>
-    <x:t>https://www.booking.com/hotel/ro/jasmine.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=17&amp;hapos=17&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=17947402_232436140_2_41_0%2C17947408_232436140_1_41_0&amp;highlighted_blocks=17947402_232436140_2_41_0%2C17947408_232436140_1_41_0&amp;matching_block_id=17947402_232436140_2_41_0&amp;sr_pri_blocks=17947402_232436140_2_41_0__4118400%2C17947408_232436140_1_41_0__2389200&amp;from=searchresults</x:t>
+    <x:t>https://www.booking.com/hotel/ro/jasmine.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=17&amp;hapos=17&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=17947402_232436140_2_41_0%2C17947408_232436140_1_41_0&amp;highlighted_blocks=17947402_232436140_2_41_0%2C17947408_232436140_1_41_0&amp;matching_block_id=17947402_232436140_2_41_0&amp;sr_pri_blocks=17947402_232436140_2_41_0__4118400%2C17947408_232436140_1_41_0__2389200&amp;from=searchresults</x:t>
   </x:si>
   <x:si>
     <x:t>Hotel Citrin - Adults Only</x:t>
@@ -265,7 +265,76 @@
     <x:t>246.8</x:t>
   </x:si>
   <x:si>
-    <x:t>https://www.booking.com/hotel/ro/citrin.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=18&amp;hapos=18&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=161216910_425257451_2_1_0%2C161216904_425257451_2_1_0&amp;highlighted_blocks=161216910_425257451_2_1_0%2C161216904_425257451_2_1_0&amp;matching_block_id=161216910_425257451_2_1_0&amp;sr_pri_blocks=161216910_425257451_2_1_0__3920400%2C161216904_425257451_2_1_0__4369200&amp;from=searchresults</x:t>
+    <x:t>https://www.booking.com/hotel/ro/citrin.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=18&amp;hapos=18&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=161216910_425257451_2_1_0%2C161216904_425257451_2_1_0&amp;highlighted_blocks=161216910_425257451_2_1_0%2C161216904_425257451_2_1_0&amp;matching_block_id=161216910_425257451_2_1_0&amp;sr_pri_blocks=161216910_425257451_2_1_0__3920400%2C161216904_425257451_2_1_0__4369200&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Hotel Oasis</x:t>
+  </x:si>
+  <x:si>
+    <x:t>136.76</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/oasis-brasov.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=19&amp;hapos=19&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=28531705_394163923_0_2_0%2C28531705_394163923_0_2_0&amp;highlighted_blocks=28531705_394163923_0_2_0%2C28531705_394163923_0_2_0&amp;matching_block_id=28531705_394163923_0_2_0&amp;sr_pri_blocks=28531705_394163923_0_2_0__2336400%2C28531705_394163923_0_2_0__2257200&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Grand Suite</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Golden Time Hotel</x:t>
+  </x:si>
+  <x:si>
+    <x:t>265.27</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8.8</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/golden-time.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=20&amp;hapos=20&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=46010206_126031212_3_1_0_1102803&amp;highlighted_blocks=46010206_126031212_3_1_0_1102803&amp;matching_block_id=46010206_126031212_3_1_0_1102803&amp;sr_pri_blocks=46010206_126031212_3_1_0_1102803_8910000&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Studio</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Galactic&amp;Ludmila Suite SPA</x:t>
+  </x:si>
+  <x:si>
+    <x:t>183.92</x:t>
+  </x:si>
+  <x:si>
+    <x:t>8.9</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/galactic.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=21&amp;hapos=21&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=1302600002_407157935_3_1_0&amp;highlighted_blocks=1302600002_407157935_3_1_0&amp;matching_block_id=1302600002_407157935_3_1_0&amp;sr_pri_blocks=1302600002_407157935_3_1_0__6177600&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>La Dolce Vita</x:t>
+  </x:si>
+  <x:si>
+    <x:t>90.12</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/la-dolce-vita-brasov.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=22&amp;hapos=22&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=1409461601_412719088_2_2_0%2C1409461602_412719088_2_2_0&amp;highlighted_blocks=1409461601_412719088_2_2_0%2C1409461602_412719088_2_2_0&amp;matching_block_id=1409461601_412719088_2_2_0&amp;sr_pri_blocks=1409461601_412719088_2_2_0__1521321%2C1409461602_412719088_2_2_0__1505513&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Hotel Regal</x:t>
+  </x:si>
+  <x:si>
+    <x:t>222.3</x:t>
+  </x:si>
+  <x:si>
+    <x:t>9.5</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/regal.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=23&amp;hapos=23&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=28949213_126030564_0_1_0_821389%2C28949205_126030564_1_1_0_821389&amp;highlighted_blocks=28949213_126030564_0_1_0_821389%2C28949205_126030564_1_1_0_821389&amp;matching_block_id=28949213_126030564_0_1_0_821389&amp;sr_pri_blocks=28949213_126030564_0_1_0_821389_3908050%2C28949205_126030564_1_1_0_821389_3559050&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Victoria Bulevard Hotel</x:t>
+  </x:si>
+  <x:si>
+    <x:t>302.61</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/victoria-bulevard-brasov.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=24&amp;hapos=24&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=212767511_126031863_2_1_0_388159%2C212767508_126031863_1_1_0_388159&amp;highlighted_blocks=212767511_126031863_2_1_0_388159%2C212767508_126031863_1_1_0_388159&amp;matching_block_id=212767511_126031863_2_1_0_388159&amp;sr_pri_blocks=212767511_126031863_2_1_0_388159_5575680%2C212767508_126031863_1_1_0_388159_4588320&amp;from=searchresults</x:t>
   </x:si>
   <x:si>
     <x:t>Stop Hotel</x:t>
@@ -277,85 +346,16 @@
     <x:t>8.5</x:t>
   </x:si>
   <x:si>
-    <x:t>https://www.booking.com/hotel/ro/stop.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=19&amp;hapos=19&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=43799104_329735434_2_2_0_1127874%2C43799104_329735434_1_2_0_1127874&amp;highlighted_blocks=43799104_329735434_2_2_0_1127874%2C43799104_329735434_1_2_0_1127874&amp;matching_block_id=43799104_329735434_2_2_0_1127874&amp;sr_pri_blocks=43799104_329735434_2_2_0_1127874_2660000%2C43799104_329735434_1_2_0_1127874_2448800&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Grand Suite</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Golden Time Hotel</x:t>
-  </x:si>
-  <x:si>
-    <x:t>265.27</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8.8</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/golden-time.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=20&amp;hapos=20&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=46010206_126031212_3_1_0_1102803&amp;highlighted_blocks=46010206_126031212_3_1_0_1102803&amp;matching_block_id=46010206_126031212_3_1_0_1102803&amp;sr_pri_blocks=46010206_126031212_3_1_0_1102803_8910000&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Studio</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Galactic&amp;Ludmila Suite SPA</x:t>
-  </x:si>
-  <x:si>
-    <x:t>183.92</x:t>
-  </x:si>
-  <x:si>
-    <x:t>8.9</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/galactic.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=21&amp;hapos=21&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=1302600002_407157935_3_1_0&amp;highlighted_blocks=1302600002_407157935_3_1_0&amp;matching_block_id=1302600002_407157935_3_1_0&amp;sr_pri_blocks=1302600002_407157935_3_1_0__6177600&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Hotel Oasis</x:t>
-  </x:si>
-  <x:si>
-    <x:t>136.76</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/oasis-brasov.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=22&amp;hapos=22&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=28531705_394163923_0_2_0%2C28531705_394163923_0_2_0&amp;highlighted_blocks=28531705_394163923_0_2_0%2C28531705_394163923_0_2_0&amp;matching_block_id=28531705_394163923_0_2_0&amp;sr_pri_blocks=28531705_394163923_0_2_0__2336400%2C28531705_394163923_0_2_0__2257200&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>La Dolce Vita</x:t>
-  </x:si>
-  <x:si>
-    <x:t>90.12</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/la-dolce-vita-brasov.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=23&amp;hapos=23&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=1409461601_412719088_2_2_0%2C1409461602_412719088_2_2_0&amp;highlighted_blocks=1409461601_412719088_2_2_0%2C1409461602_412719088_2_2_0&amp;matching_block_id=1409461601_412719088_2_2_0&amp;sr_pri_blocks=1409461601_412719088_2_2_0__1521321%2C1409461602_412719088_2_2_0__1505513&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Hotel Regal</x:t>
-  </x:si>
-  <x:si>
-    <x:t>222.3</x:t>
-  </x:si>
-  <x:si>
-    <x:t>9.5</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/regal.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=24&amp;hapos=24&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=28949213_126030564_0_1_0_821389%2C28949205_126030564_1_1_0_821389&amp;highlighted_blocks=28949213_126030564_0_1_0_821389%2C28949205_126030564_1_1_0_821389&amp;matching_block_id=28949213_126030564_0_1_0_821389&amp;sr_pri_blocks=28949213_126030564_0_1_0_821389_3908050%2C28949205_126030564_1_1_0_821389_3559050&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Victoria Bulevard Hotel</x:t>
-  </x:si>
-  <x:si>
-    <x:t>302.61</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/victoria-bulevard-brasov.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=25&amp;hapos=25&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=212767511_126031863_2_1_0_388159%2C212767508_126031863_1_1_0_388159&amp;highlighted_blocks=212767511_126031863_2_1_0_388159%2C212767508_126031863_1_1_0_388159&amp;matching_block_id=212767511_126031863_2_1_0_388159&amp;sr_pri_blocks=212767511_126031863_2_1_0_388159_5575680%2C212767508_126031863_1_1_0_388159_4588320&amp;from=searchresults</x:t>
+    <x:t>https://www.booking.com/hotel/ro/stop.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=25&amp;hapos=25&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=43799104_329735434_2_2_0_1127874%2C43799104_329735434_1_2_0_1127874&amp;highlighted_blocks=43799104_329735434_2_2_0_1127874%2C43799104_329735434_1_2_0_1127874&amp;matching_block_id=43799104_329735434_2_2_0_1127874&amp;sr_pri_blocks=43799104_329735434_2_2_0_1127874_2660000%2C43799104_329735434_1_2_0_1127874_2448800&amp;from=searchresults</x:t>
   </x:si>
   <x:si>
     <x:t>Grand Chalet Aparthotel</x:t>
   </x:si>
   <x:si>
-    <x:t>104.67</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/grand-chalet-aparthotel.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=1&amp;hapos=26&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=1252688602_397776613_3_0_0&amp;highlighted_blocks=1252688602_397776613_3_0_0&amp;matching_block_id=1252688602_397776613_3_0_0&amp;sr_pri_blocks=1252688602_397776613_3_0_0__3515375&amp;from=searchresults</x:t>
+    <x:t>105.39</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/grand-chalet-aparthotel.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=1&amp;hapos=26&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=1252688602_397776613_3_0_0&amp;highlighted_blocks=1252688602_397776613_3_0_0&amp;matching_block_id=1252688602_397776613_3_0_0&amp;sr_pri_blocks=1252688602_397776613_3_0_0__3539975&amp;from=searchresults</x:t>
   </x:si>
   <x:si>
     <x:t>Deluxe Junior Suite</x:t>
@@ -367,7 +367,7 @@
     <x:t>170.59</x:t>
   </x:si>
   <x:si>
-    <x:t>https://www.booking.com/hotel/ro/elexus-poiana-brasov.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=3&amp;hapos=28&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=721111201_309180521_0_1_0_1157365&amp;highlighted_blocks=721111201_309180521_0_1_0_1157365&amp;matching_block_id=721111201_309180521_0_1_0_1157365&amp;sr_pri_blocks=721111201_309180521_0_1_0_1157365_5729900&amp;from=searchresults</x:t>
+    <x:t>https://www.booking.com/hotel/ro/elexus-poiana-brasov.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=3&amp;hapos=28&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=721111201_309180521_0_1_0_1157365&amp;highlighted_blocks=721111201_309180521_0_1_0_1157365&amp;matching_block_id=721111201_309180521_0_1_0_1157365&amp;sr_pri_blocks=721111201_309180521_0_1_0_1157365_5729900&amp;from=searchresults</x:t>
   </x:si>
   <x:si>
     <x:t>Standard Triple Room</x:t>
@@ -379,7 +379,7 @@
     <x:t>109.26</x:t>
   </x:si>
   <x:si>
-    <x:t>https://www.booking.com/hotel/ro/condor-brasov.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=4&amp;hapos=29&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=888744704_358830520_3_2_0&amp;highlighted_blocks=888744704_358830520_3_2_0&amp;matching_block_id=888744704_358830520_3_2_0&amp;sr_pri_blocks=888744704_358830520_3_2_0__3669600&amp;from=searchresults</x:t>
+    <x:t>https://www.booking.com/hotel/ro/condor-brasov.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=4&amp;hapos=29&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=888744704_358830520_3_2_0&amp;highlighted_blocks=888744704_358830520_3_2_0&amp;matching_block_id=888744704_358830520_3_2_0&amp;sr_pri_blocks=888744704_358830520_3_2_0__3669600&amp;from=searchresults</x:t>
   </x:si>
   <x:si>
     <x:t>Silver Mountain Resort &amp; Spa</x:t>
@@ -388,7 +388,43 @@
     <x:t>212.17</x:t>
   </x:si>
   <x:si>
-    <x:t>https://www.booking.com/hotel/ro/silver-mountain-resort.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=5&amp;hapos=30&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=407154501_145154469_0_2_0_1157364%2C407154501_145154469_0_2_0_1157364&amp;highlighted_blocks=407154501_145154469_0_2_0_1157364%2C407154501_145154469_0_2_0_1157364&amp;matching_block_id=407154501_145154469_0_2_0_1157364&amp;sr_pri_blocks=407154501_145154469_0_2_0_1157364_3602800%2C407154501_145154469_0_2_0_1157364_3523600&amp;from=searchresults</x:t>
+    <x:t>https://www.booking.com/hotel/ro/silver-mountain-resort.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=5&amp;hapos=30&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=407154501_145154469_0_2_0_1157364%2C407154501_145154469_0_2_0_1157364&amp;highlighted_blocks=407154501_145154469_0_2_0_1157364%2C407154501_145154469_0_2_0_1157364&amp;matching_block_id=407154501_145154469_0_2_0_1157364&amp;sr_pri_blocks=407154501_145154469_0_2_0_1157364_3602800%2C407154501_145154469_0_2_0_1157364_3523600&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Premont Luxury Ghimbav</x:t>
+  </x:si>
+  <x:si>
+    <x:t>105.76</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/premont-luxury-ghimbav.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=6&amp;hapos=31&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=1356501001_407981561_2_0_0%2C1356501002_408301105_0_0_0&amp;highlighted_blocks=1356501001_407981561_2_0_0%2C1356501002_408301105_0_0_0&amp;matching_block_id=1356501001_407981561_2_0_0&amp;sr_pri_blocks=1356501001_407981561_2_0_0__1639440%2C1356501002_408301105_0_0_0__1912680&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Superior Two-Bedroom Suite</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Hotel Miruna - New Belvedere</x:t>
+  </x:si>
+  <x:si>
+    <x:t>276.27</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/miruna-poiana-brasov.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=7&amp;hapos=32&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=36759405_126031009_0_1_0&amp;highlighted_blocks=36759405_126031009_0_1_0&amp;matching_block_id=36759405_126031009_0_1_0&amp;sr_pri_blocks=36759405_126031009_0_1_0__9279600&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Two-Bedroom Apartment</x:t>
+  </x:si>
+  <x:si>
+    <x:t>HOTEL ALL TIMES</x:t>
+  </x:si>
+  <x:si>
+    <x:t>59.03</x:t>
+  </x:si>
+  <x:si>
+    <x:t>7.0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/all-times-timisul-de-jos.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=8&amp;hapos=33&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=667401303_273255331_3_0_0&amp;highlighted_blocks=667401303_273255331_3_0_0&amp;matching_block_id=667401303_273255331_3_0_0&amp;sr_pri_blocks=667401303_273255331_3_0_0__1982600&amp;from=searchresults</x:t>
   </x:si>
   <x:si>
     <x:t>One-Bedroom Deluxe Apartment</x:t>
@@ -400,43 +436,7 @@
     <x:t>48.8</x:t>
   </x:si>
   <x:si>
-    <x:t>https://www.booking.com/hotel/ro/premont-studios-ghimbav.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=6&amp;hapos=31&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=858979004_362697679_3_0_0&amp;highlighted_blocks=858979004_362697679_3_0_0&amp;matching_block_id=858979004_362697679_3_0_0&amp;sr_pri_blocks=858979004_362697679_3_0_0__1639440&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Premont Luxury Ghimbav</x:t>
-  </x:si>
-  <x:si>
-    <x:t>105.76</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/premont-luxury-ghimbav.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=7&amp;hapos=32&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=1356501001_407981561_2_0_0%2C1356501002_408301105_0_0_0&amp;highlighted_blocks=1356501001_407981561_2_0_0%2C1356501002_408301105_0_0_0&amp;matching_block_id=1356501001_407981561_2_0_0&amp;sr_pri_blocks=1356501001_407981561_2_0_0__1639440%2C1356501002_408301105_0_0_0__1912680&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Superior Two-Bedroom Suite</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Hotel Miruna - New Belvedere</x:t>
-  </x:si>
-  <x:si>
-    <x:t>276.27</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/miruna-poiana-brasov.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=8&amp;hapos=33&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=36759405_126031009_0_1_0&amp;highlighted_blocks=36759405_126031009_0_1_0&amp;matching_block_id=36759405_126031009_0_1_0&amp;sr_pri_blocks=36759405_126031009_0_1_0__9279600&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Two-Bedroom Apartment</x:t>
-  </x:si>
-  <x:si>
-    <x:t>HOTEL ALL TIMES</x:t>
-  </x:si>
-  <x:si>
-    <x:t>59.03</x:t>
-  </x:si>
-  <x:si>
-    <x:t>7.0</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/all-times-timisul-de-jos.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=9&amp;hapos=34&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=667401303_273255331_3_0_0&amp;highlighted_blocks=667401303_273255331_3_0_0&amp;matching_block_id=667401303_273255331_3_0_0&amp;sr_pri_blocks=667401303_273255331_3_0_0__1982600&amp;from=searchresults</x:t>
+    <x:t>https://www.booking.com/hotel/ro/premont-studios-ghimbav.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=9&amp;hapos=34&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=858979004_362697679_3_0_0&amp;highlighted_blocks=858979004_362697679_3_0_0&amp;matching_block_id=858979004_362697679_3_0_0&amp;sr_pri_blocks=858979004_362697679_3_0_0__1639440&amp;from=searchresults</x:t>
   </x:si>
   <x:si>
     <x:t>Alpin Resort Hotel - Apartamentele 2403-2404- proprietate administrata de gazda privata</x:t>
@@ -445,7 +445,7 @@
     <x:t>240.91</x:t>
   </x:si>
   <x:si>
-    <x:t>https://www.booking.com/hotel/ro/alpin-resort-apartament-2403-2404.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=10&amp;hapos=35&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=753323001_331951697_0_1_0&amp;highlighted_blocks=753323001_331951697_0_1_0&amp;matching_block_id=753323001_331951697_0_1_0&amp;sr_pri_blocks=753323001_331951697_0_1_0__8091600&amp;from=searchresults</x:t>
+    <x:t>https://www.booking.com/hotel/ro/alpin-resort-apartament-2403-2404.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=10&amp;hapos=35&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=753323001_331951697_0_1_0&amp;highlighted_blocks=753323001_331951697_0_1_0&amp;matching_block_id=753323001_331951697_0_1_0&amp;sr_pri_blocks=753323001_331951697_0_1_0__8091600&amp;from=searchresults</x:t>
   </x:si>
   <x:si>
     <x:t>Alpin Resort Apartments Deluxe 2406</x:t>
@@ -454,7 +454,7 @@
     <x:t>272.33</x:t>
   </x:si>
   <x:si>
-    <x:t>https://www.booking.com/hotel/ro/alpin-resort-deluxe-apartment.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=11&amp;hapos=36&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=865725401_354756822_4_2_0&amp;highlighted_blocks=865725401_354756822_4_2_0&amp;matching_block_id=865725401_354756822_4_2_0&amp;sr_pri_blocks=865725401_354756822_4_2_0__9147600&amp;from=searchresults</x:t>
+    <x:t>https://www.booking.com/hotel/ro/alpin-resort-deluxe-apartment.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=11&amp;hapos=36&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=865725401_354756822_4_2_0&amp;highlighted_blocks=865725401_354756822_4_2_0&amp;matching_block_id=865725401_354756822_4_2_0&amp;sr_pri_blocks=865725401_354756822_4_2_0__9147600&amp;from=searchresults</x:t>
   </x:si>
   <x:si>
     <x:t>Superior Apartment</x:t>
@@ -466,7 +466,7 @@
     <x:t>284.68</x:t>
   </x:si>
   <x:si>
-    <x:t>https://www.booking.com/hotel/ro/alpin-resort-aparthotel.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=12&amp;hapos=37&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=707480101_418566801_0_0_0_808194&amp;highlighted_blocks=707480101_418566801_0_0_0_808194&amp;matching_block_id=707480101_418566801_0_0_0_808194&amp;sr_pri_blocks=707480101_418566801_0_0_0_808194_9561900&amp;from=searchresults</x:t>
+    <x:t>https://www.booking.com/hotel/ro/alpin-resort-aparthotel.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=12&amp;hapos=37&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=707480101_418566801_0_0_0_808194&amp;highlighted_blocks=707480101_418566801_0_0_0_808194&amp;matching_block_id=707480101_418566801_0_0_0_808194&amp;sr_pri_blocks=707480101_418566801_0_0_0_808194_9561900&amp;from=searchresults</x:t>
   </x:si>
   <x:si>
     <x:t>Hotel Piemonte</x:t>
@@ -478,7 +478,7 @@
     <x:t>8.4</x:t>
   </x:si>
   <x:si>
-    <x:t>https://www.booking.com/hotel/ro/piemonte.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=13&amp;hapos=38&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=17861431_128927040_0_2_0%2C17861431_128927040_1_2_0&amp;highlighted_blocks=17861431_128927040_0_2_0%2C17861431_128927040_1_2_0&amp;matching_block_id=17861431_128927040_0_2_0&amp;sr_pri_blocks=17861431_128927040_0_2_0__1677528%2C17861431_128927040_1_2_0__1269738&amp;from=searchresults</x:t>
+    <x:t>https://www.booking.com/hotel/ro/piemonte.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=13&amp;hapos=38&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=17861431_128927040_0_2_0%2C17861431_128927040_1_2_0&amp;highlighted_blocks=17861431_128927040_0_2_0%2C17861431_128927040_1_2_0&amp;matching_block_id=17861431_128927040_0_2_0&amp;sr_pri_blocks=17861431_128927040_0_2_0__1677528%2C17861431_128927040_1_2_0__1269738&amp;from=searchresults</x:t>
   </x:si>
   <x:si>
     <x:t>Suite</x:t>
@@ -490,7 +490,7 @@
     <x:t>108.39</x:t>
   </x:si>
   <x:si>
-    <x:t>https://www.booking.com/hotel/ro/belvedere-predeal.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=14&amp;hapos=39&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=48485603_126031242_0_1_0&amp;highlighted_blocks=48485603_126031242_0_1_0&amp;matching_block_id=48485603_126031242_0_1_0&amp;sr_pri_blocks=48485603_126031242_0_1_0__3641000&amp;from=searchresults</x:t>
+    <x:t>https://www.booking.com/hotel/ro/belvedere-predeal.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=14&amp;hapos=39&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=48485603_126031242_0_1_0&amp;highlighted_blocks=48485603_126031242_0_1_0&amp;matching_block_id=48485603_126031242_0_1_0&amp;sr_pri_blocks=48485603_126031242_0_1_0__3641000&amp;from=searchresults</x:t>
   </x:si>
   <x:si>
     <x:t>Cabana Trei Brazi</x:t>
@@ -499,7 +499,7 @@
     <x:t>112.98</x:t>
   </x:si>
   <x:si>
-    <x:t>https://www.booking.com/hotel/ro/cabana-trei-brazi.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=15&amp;hapos=40&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=36951801_126031062_0_0_0%2C36951801_126031062_0_0_0&amp;highlighted_blocks=36951801_126031062_0_0_0%2C36951801_126031062_0_0_0&amp;matching_block_id=36951801_126031062_0_0_0&amp;sr_pri_blocks=36951801_126031062_0_0_0__1914000%2C36951801_126031062_0_0_0__1881000&amp;from=searchresults</x:t>
+    <x:t>https://www.booking.com/hotel/ro/cabana-trei-brazi.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=15&amp;hapos=40&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=36951801_126031062_0_0_0%2C36951801_126031062_0_0_0&amp;highlighted_blocks=36951801_126031062_0_0_0%2C36951801_126031062_0_0_0&amp;matching_block_id=36951801_126031062_0_0_0&amp;sr_pri_blocks=36951801_126031062_0_0_0__1914000%2C36951801_126031062_0_0_0__1881000&amp;from=searchresults</x:t>
   </x:si>
   <x:si>
     <x:t>Junior Suite</x:t>
@@ -511,7 +511,7 @@
     <x:t>130.64</x:t>
   </x:si>
   <x:si>
-    <x:t>https://www.booking.com/hotel/ro/elexus-boutique.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=16&amp;hapos=41&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=623385106_401381041_3_1_0_690170&amp;highlighted_blocks=623385106_401381041_3_1_0_690170&amp;matching_block_id=623385106_401381041_3_1_0_690170&amp;sr_pri_blocks=623385106_401381041_3_1_0_690170_4388040&amp;from=searchresults</x:t>
+    <x:t>https://www.booking.com/hotel/ro/elexus-boutique.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=16&amp;hapos=41&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=623385106_401381041_3_1_0_690170&amp;highlighted_blocks=623385106_401381041_3_1_0_690170&amp;matching_block_id=623385106_401381041_3_1_0_690170&amp;sr_pri_blocks=623385106_401381041_3_1_0_690170_4388040&amp;from=searchresults</x:t>
   </x:si>
   <x:si>
     <x:t>Apartment with Free Infinity Pool access</x:t>
@@ -523,7 +523,19 @@
     <x:t>220.83</x:t>
   </x:si>
   <x:si>
-    <x:t>https://www.booking.com/hotel/ro/elexus-predeal.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=17&amp;hapos=42&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=628026602_401381023_3_1_0_843076&amp;highlighted_blocks=628026602_401381023_3_1_0_843076&amp;matching_block_id=628026602_401381023_3_1_0_843076&amp;sr_pri_blocks=628026602_401381023_3_1_0_843076_7417600&amp;from=searchresults</x:t>
+    <x:t>https://www.booking.com/hotel/ro/elexus-predeal.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=17&amp;hapos=42&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=628026602_401381023_3_1_0_843076&amp;highlighted_blocks=628026602_401381023_3_1_0_843076&amp;matching_block_id=628026602_401381023_3_1_0_843076&amp;sr_pri_blocks=628026602_401381023_3_1_0_843076_7417600&amp;from=searchresults</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Apartment with Garden View</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Cedar Crest</x:t>
+  </x:si>
+  <x:si>
+    <x:t>168</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/cedar-crest.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=18&amp;hapos=43&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=595133301_233514441_6_0_0&amp;highlighted_blocks=595133301_233514441_6_0_0&amp;matching_block_id=595133301_233514441_6_0_0&amp;sr_pri_blocks=595133301_233514441_6_0_0__5643000&amp;from=searchresults</x:t>
   </x:si>
   <x:si>
     <x:t>Hotel Express</x:t>
@@ -532,28 +544,16 @@
     <x:t>8.7</x:t>
   </x:si>
   <x:si>
-    <x:t>https://www.booking.com/hotel/ro/express.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=18&amp;hapos=43&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=90240201_347651904_2_1_0_220738%2C90240201_347651904_2_1_0_220738&amp;highlighted_blocks=90240201_347651904_2_1_0_220738%2C90240201_347651904_2_1_0_220738&amp;matching_block_id=90240201_347651904_2_1_0_220738&amp;sr_pri_blocks=90240201_347651904_2_1_0_220738_1914000%2C90240201_347651904_2_1_0_220738_1881000&amp;from=searchresults</x:t>
+    <x:t>https://www.booking.com/hotel/ro/express.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=19&amp;hapos=44&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=90240201_347651904_2_1_0_220738%2C90240201_347651904_2_1_0_220738&amp;highlighted_blocks=90240201_347651904_2_1_0_220738%2C90240201_347651904_2_1_0_220738&amp;matching_block_id=90240201_347651904_2_1_0_220738&amp;sr_pri_blocks=90240201_347651904_2_1_0_220738_1914000%2C90240201_347651904_2_1_0_220738_1881000&amp;from=searchresults</x:t>
   </x:si>
   <x:si>
     <x:t>Voila Inn Predeal</x:t>
   </x:si>
   <x:si>
-    <x:t>137.35</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/voila-inn-predeal.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=19&amp;hapos=44&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=839479501_350509506_0_1_0&amp;highlighted_blocks=839479501_350509506_0_1_0&amp;matching_block_id=839479501_350509506_0_1_0&amp;sr_pri_blocks=839479501_350509506_0_1_0__4613400&amp;from=searchresults</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Apartment with Garden View</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Cedar Crest</x:t>
-  </x:si>
-  <x:si>
-    <x:t>168</x:t>
-  </x:si>
-  <x:si>
-    <x:t>https://www.booking.com/hotel/ro/cedar-crest.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=20&amp;hapos=45&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=595133301_233514441_6_0_0&amp;highlighted_blocks=595133301_233514441_6_0_0&amp;matching_block_id=595133301_233514441_6_0_0&amp;sr_pri_blocks=595133301_233514441_6_0_0__5643000&amp;from=searchresults</x:t>
+    <x:t>152.29</x:t>
+  </x:si>
+  <x:si>
+    <x:t>https://www.booking.com/hotel/ro/voila-inn-predeal.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=20&amp;hapos=45&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=839479501_350509506_0_1_0&amp;highlighted_blocks=839479501_350509506_0_1_0&amp;matching_block_id=839479501_350509506_0_1_0&amp;sr_pri_blocks=839479501_350509506_0_1_0__5115000&amp;from=searchresults</x:t>
   </x:si>
   <x:si>
     <x:t>New Wolf</x:t>
@@ -562,7 +562,7 @@
     <x:t>177.27</x:t>
   </x:si>
   <x:si>
-    <x:t>https://www.booking.com/hotel/ro/wolf-1.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=21&amp;hapos=46&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=25972803_127405559_0_0_0_76049%2C25972803_127405559_0_0_0_76049&amp;highlighted_blocks=25972803_127405559_0_0_0_76049%2C25972803_127405559_0_0_0_76049&amp;matching_block_id=25972803_127405559_0_0_0_76049&amp;sr_pri_blocks=25972803_127405559_0_0_0_76049_2977100%2C25972803_127405559_0_0_0_76049_2977100&amp;from=searchresults</x:t>
+    <x:t>https://www.booking.com/hotel/ro/wolf-1.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=21&amp;hapos=46&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=25972803_127405559_0_0_0_76049%2C25972803_127405559_0_0_0_76049&amp;highlighted_blocks=25972803_127405559_0_0_0_76049%2C25972803_127405559_0_0_0_76049&amp;matching_block_id=25972803_127405559_0_0_0_76049&amp;sr_pri_blocks=25972803_127405559_0_0_0_76049_2977100%2C25972803_127405559_0_0_0_76049_2977100&amp;from=searchresults</x:t>
   </x:si>
   <x:si>
     <x:t>Gura Diham</x:t>
@@ -571,7 +571,7 @@
     <x:t>110.06</x:t>
   </x:si>
   <x:si>
-    <x:t>https://www.booking.com/hotel/ro/gura-diham.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKDko7LBsACAdICJGQ0YmQ3OTk5LWY4YjAtNDZhMC05Y2ViLTBkZGM2Njc5YmJkNtgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=22&amp;hapos=47&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=649e225ec1cc84298ca0a0539fc9c3a5&amp;srepoch=1768130844&amp;all_sr_blocks=44344301_329736299_2_0_0%2C44344301_329736299_2_0_0&amp;highlighted_blocks=44344301_329736299_2_0_0%2C44344301_329736299_2_0_0&amp;matching_block_id=44344301_329736299_2_0_0&amp;sr_pri_blocks=44344301_329736299_2_0_0__1848600%2C44344301_329736299_2_0_0__1848300&amp;from=searchresults</x:t>
+    <x:t>https://www.booking.com/hotel/ro/gura-diham.html?label=gen173bo-10CAEoggI46AdIM1gDaMABiAEBmAEzuAEXyAEM2AED6AEB-AEBiAIBmAICqAIBuAKVr47LBsACAdICJDY1OGI2N2I1LTYzNjktNDQ4My05NDQ2LWRiNjQyZTBiMGY0MdgCAeACAQ&amp;aid=304142&amp;ucfs=1&amp;arphpl=1&amp;checkin=2026-05-15&amp;checkout=2026-07-20&amp;dest_id=-1153613&amp;dest_type=city&amp;group_adults=3&amp;req_adults=3&amp;no_rooms=1&amp;group_children=0&amp;req_children=0&amp;hpos=22&amp;hapos=47&amp;sr_order=popularity&amp;nflt=ht_id%3D204&amp;srpvid=cef9740df7dc47c80b3ab66496cb54d4&amp;srepoch=1768134572&amp;all_sr_blocks=44344301_329736299_2_0_0%2C44344301_329736299_2_0_0&amp;highlighted_blocks=44344301_329736299_2_0_0%2C44344301_329736299_2_0_0&amp;matching_block_id=44344301_329736299_2_0_0&amp;sr_pri_blocks=44344301_329736299_2_0_0__1848600%2C44344301_329736299_2_0_0__1848300&amp;from=searchresults</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1039,10 +1039,10 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F6" s="0" t="s">
         <x:v>30</x:v>
-      </x:c>
-      <x:c r="F6" s="0" t="s">
-        <x:v>31</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:6">
@@ -1050,19 +1050,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="C7" s="0" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="C7" s="0" t="s">
+      <x:c r="D7" s="0" t="s">
         <x:v>33</x:v>
       </x:c>
-      <x:c r="D7" s="0" t="s">
+      <x:c r="E7" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="F7" s="0" t="s">
         <x:v>34</x:v>
-      </x:c>
-      <x:c r="E7" s="0" t="s">
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="F7" s="0" t="s">
-        <x:v>35</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:6">
@@ -1070,19 +1070,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
         <x:v>36</x:v>
       </x:c>
-      <x:c r="C8" s="0" t="s">
+      <x:c r="D8" s="0" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="D8" s="0" t="s">
+      <x:c r="E8" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F8" s="0" t="s">
         <x:v>38</x:v>
-      </x:c>
-      <x:c r="E8" s="0" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="F8" s="0" t="s">
-        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:6">
@@ -1090,19 +1090,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="C9" s="0" t="s">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="D9" s="0" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="C9" s="0" t="s">
+      <x:c r="E9" s="0" t="s">
         <x:v>42</x:v>
       </x:c>
-      <x:c r="D9" s="0" t="s">
+      <x:c r="F9" s="0" t="s">
         <x:v>43</x:v>
-      </x:c>
-      <x:c r="E9" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="F9" s="0" t="s">
-        <x:v>44</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:6">
@@ -1110,19 +1110,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B10" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C10" s="0" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="D10" s="0" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="C10" s="0" t="s">
+      <x:c r="E10" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F10" s="0" t="s">
         <x:v>46</x:v>
-      </x:c>
-      <x:c r="D10" s="0" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="E10" s="0" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="F10" s="0" t="s">
-        <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:6">
@@ -1130,19 +1130,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B11" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C11" s="0" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="D11" s="0" t="s">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="E11" s="0" t="s">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F11" s="0" t="s">
         <x:v>50</x:v>
-      </x:c>
-      <x:c r="D11" s="0" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E11" s="0" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="F11" s="0" t="s">
-        <x:v>52</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:6">
@@ -1150,19 +1150,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B12" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C12" s="0" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="D12" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="E12" s="0" t="s">
         <x:v>53</x:v>
       </x:c>
-      <x:c r="C12" s="0" t="s">
+      <x:c r="F12" s="0" t="s">
         <x:v>54</x:v>
-      </x:c>
-      <x:c r="D12" s="0" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="E12" s="0" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="F12" s="0" t="s">
-        <x:v>56</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:6">
@@ -1170,19 +1170,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B13" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C13" s="0" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="D13" s="0" t="s">
         <x:v>57</x:v>
       </x:c>
-      <x:c r="D13" s="0" t="s">
+      <x:c r="E13" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="F13" s="0" t="s">
         <x:v>58</x:v>
-      </x:c>
-      <x:c r="E13" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="F13" s="0" t="s">
-        <x:v>59</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:6">
@@ -1190,19 +1190,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B14" s="0" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="C14" s="0" t="s">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="C14" s="0" t="s">
+      <x:c r="D14" s="0" t="s">
         <x:v>61</x:v>
       </x:c>
-      <x:c r="D14" s="0" t="s">
+      <x:c r="E14" s="0" t="s">
         <x:v>62</x:v>
       </x:c>
-      <x:c r="E14" s="0" t="s">
+      <x:c r="F14" s="0" t="s">
         <x:v>63</x:v>
-      </x:c>
-      <x:c r="F14" s="0" t="s">
-        <x:v>64</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:6">
@@ -1210,19 +1210,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B15" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C15" s="0" t="s">
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="D15" s="0" t="s">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="D15" s="0" t="s">
+      <x:c r="E15" s="0" t="s">
         <x:v>66</x:v>
       </x:c>
-      <x:c r="E15" s="0" t="s">
+      <x:c r="F15" s="0" t="s">
         <x:v>67</x:v>
-      </x:c>
-      <x:c r="F15" s="0" t="s">
-        <x:v>68</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:6">
@@ -1230,19 +1230,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B16" s="0" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="C16" s="0" t="s">
         <x:v>69</x:v>
       </x:c>
-      <x:c r="C16" s="0" t="s">
+      <x:c r="D16" s="0" t="s">
         <x:v>70</x:v>
       </x:c>
-      <x:c r="D16" s="0" t="s">
+      <x:c r="E16" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="F16" s="0" t="s">
         <x:v>71</x:v>
-      </x:c>
-      <x:c r="E16" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="F16" s="0" t="s">
-        <x:v>72</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:6">
@@ -1250,16 +1250,16 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B17" s="0" t="s">
+        <x:v>72</x:v>
+      </x:c>
+      <x:c r="C17" s="0" t="s">
         <x:v>73</x:v>
       </x:c>
-      <x:c r="C17" s="0" t="s">
+      <x:c r="D17" s="0" t="s">
         <x:v>74</x:v>
       </x:c>
-      <x:c r="D17" s="0" t="s">
+      <x:c r="E17" s="0" t="s">
         <x:v>75</x:v>
-      </x:c>
-      <x:c r="E17" s="0" t="s">
-        <x:v>20</x:v>
       </x:c>
       <x:c r="F17" s="0" t="s">
         <x:v>76</x:v>
@@ -1270,7 +1270,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B18" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C18" s="0" t="s">
         <x:v>77</x:v>
@@ -1290,7 +1290,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B19" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C19" s="0" t="s">
         <x:v>81</x:v>
@@ -1299,7 +1299,7 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="E19" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F19" s="0" t="s">
         <x:v>83</x:v>
@@ -1310,7 +1310,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B20" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C20" s="0" t="s">
         <x:v>84</x:v>
@@ -1319,10 +1319,10 @@
         <x:v>85</x:v>
       </x:c>
       <x:c r="E20" s="0" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="F20" s="0" t="s">
         <x:v>86</x:v>
-      </x:c>
-      <x:c r="F20" s="0" t="s">
-        <x:v>87</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:6">
@@ -1330,19 +1330,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B21" s="0" t="s">
+        <x:v>87</x:v>
+      </x:c>
+      <x:c r="C21" s="0" t="s">
         <x:v>88</x:v>
       </x:c>
-      <x:c r="C21" s="0" t="s">
+      <x:c r="D21" s="0" t="s">
         <x:v>89</x:v>
       </x:c>
-      <x:c r="D21" s="0" t="s">
+      <x:c r="E21" s="0" t="s">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="E21" s="0" t="s">
+      <x:c r="F21" s="0" t="s">
         <x:v>91</x:v>
-      </x:c>
-      <x:c r="F21" s="0" t="s">
-        <x:v>92</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:6">
@@ -1350,19 +1350,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B22" s="0" t="s">
+        <x:v>92</x:v>
+      </x:c>
+      <x:c r="C22" s="0" t="s">
         <x:v>93</x:v>
       </x:c>
-      <x:c r="C22" s="0" t="s">
+      <x:c r="D22" s="0" t="s">
         <x:v>94</x:v>
       </x:c>
-      <x:c r="D22" s="0" t="s">
+      <x:c r="E22" s="0" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="E22" s="0" t="s">
+      <x:c r="F22" s="0" t="s">
         <x:v>96</x:v>
-      </x:c>
-      <x:c r="F22" s="0" t="s">
-        <x:v>97</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:6">
@@ -1370,19 +1370,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B23" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C23" s="0" t="s">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="D23" s="0" t="s">
         <x:v>98</x:v>
       </x:c>
-      <x:c r="D23" s="0" t="s">
+      <x:c r="E23" s="0" t="s">
+        <x:v>95</x:v>
+      </x:c>
+      <x:c r="F23" s="0" t="s">
         <x:v>99</x:v>
-      </x:c>
-      <x:c r="E23" s="0" t="s">
-        <x:v>63</x:v>
-      </x:c>
-      <x:c r="F23" s="0" t="s">
-        <x:v>100</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:6">
@@ -1390,16 +1390,16 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B24" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C24" s="0" t="s">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="D24" s="0" t="s">
         <x:v>101</x:v>
       </x:c>
-      <x:c r="D24" s="0" t="s">
+      <x:c r="E24" s="0" t="s">
         <x:v>102</x:v>
-      </x:c>
-      <x:c r="E24" s="0" t="s">
-        <x:v>96</x:v>
       </x:c>
       <x:c r="F24" s="0" t="s">
         <x:v>103</x:v>
@@ -1410,7 +1410,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B25" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C25" s="0" t="s">
         <x:v>104</x:v>
@@ -1419,10 +1419,10 @@
         <x:v>105</x:v>
       </x:c>
       <x:c r="E25" s="0" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="F25" s="0" t="s">
         <x:v>106</x:v>
-      </x:c>
-      <x:c r="F25" s="0" t="s">
-        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:6">
@@ -1430,16 +1430,16 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B26" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C26" s="0" t="s">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="D26" s="0" t="s">
         <x:v>108</x:v>
       </x:c>
-      <x:c r="D26" s="0" t="s">
+      <x:c r="E26" s="0" t="s">
         <x:v>109</x:v>
-      </x:c>
-      <x:c r="E26" s="0" t="s">
-        <x:v>67</x:v>
       </x:c>
       <x:c r="F26" s="0" t="s">
         <x:v>110</x:v>
@@ -1450,7 +1450,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B27" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C27" s="0" t="s">
         <x:v>111</x:v>
@@ -1459,7 +1459,7 @@
         <x:v>112</x:v>
       </x:c>
       <x:c r="E27" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F27" s="0" t="s">
         <x:v>113</x:v>
@@ -1479,7 +1479,7 @@
         <x:v>116</x:v>
       </x:c>
       <x:c r="E28" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="F28" s="0" t="s">
         <x:v>117</x:v>
@@ -1499,7 +1499,7 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="E29" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="F29" s="0" t="s">
         <x:v>121</x:v>
@@ -1510,7 +1510,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B30" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C30" s="0" t="s">
         <x:v>122</x:v>
@@ -1519,7 +1519,7 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="E30" s="0" t="s">
-        <x:v>96</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="F30" s="0" t="s">
         <x:v>124</x:v>
@@ -1530,19 +1530,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B31" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="C31" s="0" t="s">
         <x:v>125</x:v>
       </x:c>
-      <x:c r="C31" s="0" t="s">
+      <x:c r="D31" s="0" t="s">
         <x:v>126</x:v>
       </x:c>
-      <x:c r="D31" s="0" t="s">
+      <x:c r="E31" s="0" t="s">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="F31" s="0" t="s">
         <x:v>127</x:v>
-      </x:c>
-      <x:c r="E31" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="F31" s="0" t="s">
-        <x:v>128</x:v>
       </x:c>
     </x:row>
     <x:row r="32" spans="1:6">
@@ -1550,7 +1550,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B32" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="C32" s="0" t="s">
         <x:v>129</x:v>
@@ -1559,7 +1559,7 @@
         <x:v>130</x:v>
       </x:c>
       <x:c r="E32" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="F32" s="0" t="s">
         <x:v>131</x:v>
@@ -1579,10 +1579,10 @@
         <x:v>134</x:v>
       </x:c>
       <x:c r="E33" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="F33" s="0" t="s">
-        <x:v>135</x:v>
+        <x:v>136</x:v>
       </x:c>
     </x:row>
     <x:row r="34" spans="1:6">
@@ -1590,16 +1590,16 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B34" s="0" t="s">
-        <x:v>136</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="C34" s="0" t="s">
-        <x:v>137</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="D34" s="0" t="s">
-        <x:v>138</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="E34" s="0" t="s">
-        <x:v>139</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="F34" s="0" t="s">
         <x:v>140</x:v>
@@ -1610,7 +1610,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B35" s="0" t="s">
-        <x:v>136</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="C35" s="0" t="s">
         <x:v>141</x:v>
@@ -1619,7 +1619,7 @@
         <x:v>142</x:v>
       </x:c>
       <x:c r="E35" s="0" t="s">
-        <x:v>106</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="F35" s="0" t="s">
         <x:v>143</x:v>
@@ -1630,7 +1630,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B36" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C36" s="0" t="s">
         <x:v>144</x:v>
@@ -1639,7 +1639,7 @@
         <x:v>145</x:v>
       </x:c>
       <x:c r="E36" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F36" s="0" t="s">
         <x:v>146</x:v>
@@ -1659,7 +1659,7 @@
         <x:v>149</x:v>
       </x:c>
       <x:c r="E37" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F37" s="0" t="s">
         <x:v>150</x:v>
@@ -1670,7 +1670,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B38" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C38" s="0" t="s">
         <x:v>151</x:v>
@@ -1699,7 +1699,7 @@
         <x:v>157</x:v>
       </x:c>
       <x:c r="E39" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="F39" s="0" t="s">
         <x:v>158</x:v>
@@ -1710,7 +1710,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B40" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C40" s="0" t="s">
         <x:v>159</x:v>
@@ -1719,7 +1719,7 @@
         <x:v>160</x:v>
       </x:c>
       <x:c r="E40" s="0" t="s">
-        <x:v>86</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="F40" s="0" t="s">
         <x:v>161</x:v>
@@ -1739,7 +1739,7 @@
         <x:v>164</x:v>
       </x:c>
       <x:c r="E41" s="0" t="s">
-        <x:v>67</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="F41" s="0" t="s">
         <x:v>165</x:v>
@@ -1759,7 +1759,7 @@
         <x:v>168</x:v>
       </x:c>
       <x:c r="E42" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="F42" s="0" t="s">
         <x:v>169</x:v>
@@ -1770,19 +1770,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B43" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="C43" s="0" t="s">
-        <x:v>170</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="D43" s="0" t="s">
-        <x:v>160</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="E43" s="0" t="s">
-        <x:v>171</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="F43" s="0" t="s">
-        <x:v>172</x:v>
+        <x:v>173</x:v>
       </x:c>
     </x:row>
     <x:row r="44" spans="1:6">
@@ -1793,16 +1793,16 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="C44" s="0" t="s">
-        <x:v>173</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="D44" s="0" t="s">
-        <x:v>174</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="E44" s="0" t="s">
-        <x:v>96</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="F44" s="0" t="s">
-        <x:v>175</x:v>
+        <x:v>176</x:v>
       </x:c>
     </x:row>
     <x:row r="45" spans="1:6">
@@ -1810,7 +1810,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B45" s="0" t="s">
-        <x:v>176</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C45" s="0" t="s">
         <x:v>177</x:v>
@@ -1819,7 +1819,7 @@
         <x:v>178</x:v>
       </x:c>
       <x:c r="E45" s="0" t="s">
-        <x:v>79</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="F45" s="0" t="s">
         <x:v>179</x:v>
@@ -1830,7 +1830,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B46" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C46" s="0" t="s">
         <x:v>180</x:v>
@@ -1839,7 +1839,7 @@
         <x:v>181</x:v>
       </x:c>
       <x:c r="E46" s="0" t="s">
-        <x:v>20</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="F46" s="0" t="s">
         <x:v>182</x:v>
@@ -1850,7 +1850,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B47" s="0" t="s">
-        <x:v>22</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C47" s="0" t="s">
         <x:v>183</x:v>
@@ -1859,7 +1859,7 @@
         <x:v>184</x:v>
       </x:c>
       <x:c r="E47" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="F47" s="0" t="s">
         <x:v>185</x:v>

</xml_diff>